<commit_message>
ALSN AOS cleaned ready
</commit_message>
<xml_diff>
--- a/alns_aos_table8_table14_seed_results.xlsx
+++ b/alns_aos_table8_table14_seed_results.xlsx
@@ -440,7 +440,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
@@ -540,7 +540,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.00054168701171875</v>
+        <v>0.0002346038818359375</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -552,14 +552,14 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3562982082366943</v>
+        <v>0.3464779853820801</v>
       </c>
       <c r="K2" t="n">
         <v>500</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -589,7 +589,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0001051425933837891</v>
+        <v>0.0001115798950195312</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -601,14 +601,14 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.3048374652862549</v>
+        <v>0.329235315322876</v>
       </c>
       <c r="K3" t="n">
         <v>500</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -638,7 +638,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0001058578491210938</v>
+        <v>0.0001761913299560547</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -650,14 +650,14 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3464863300323486</v>
+        <v>0.4010365009307861</v>
       </c>
       <c r="K4" t="n">
         <v>500</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -687,7 +687,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0001058578491210938</v>
+        <v>0.0001339912414550781</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -699,14 +699,14 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3205859661102295</v>
+        <v>0.3659090995788574</v>
       </c>
       <c r="K5" t="n">
         <v>500</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -736,7 +736,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0001189708709716797</v>
+        <v>0.0001704692840576172</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -748,14 +748,14 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3028337955474854</v>
+        <v>0.39713454246521</v>
       </c>
       <c r="K6" t="n">
         <v>500</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -785,7 +785,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0001461505889892578</v>
+        <v>0.0001964569091796875</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -797,14 +797,14 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3493485450744629</v>
+        <v>0.4668540954589844</v>
       </c>
       <c r="K7" t="n">
         <v>500</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0001046657562255859</v>
+        <v>0.0002582073211669922</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -846,14 +846,14 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3332276344299316</v>
+        <v>0.394345760345459</v>
       </c>
       <c r="K8" t="n">
         <v>500</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -883,7 +883,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0001175403594970703</v>
+        <v>0.0001063346862792969</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -895,14 +895,14 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3223223686218262</v>
+        <v>0.4503626823425293</v>
       </c>
       <c r="K9" t="n">
         <v>500</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0001215934753417969</v>
+        <v>0.0004088878631591797</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -944,14 +944,14 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.3009412288665771</v>
+        <v>0.4266672134399414</v>
       </c>
       <c r="K10" t="n">
         <v>500</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -981,7 +981,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0001592636108398438</v>
+        <v>0.0001156330108642578</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -993,14 +993,14 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.3577518463134766</v>
+        <v>0.464343786239624</v>
       </c>
       <c r="K11" t="n">
         <v>500</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0002193450927734375</v>
+        <v>0.0002546310424804688</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -1042,14 +1042,14 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.9003226757049561</v>
+        <v>1.093500375747681</v>
       </c>
       <c r="K12" t="n">
         <v>500</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1079,7 +1079,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0001785755157470703</v>
+        <v>0.0001769065856933594</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -1091,14 +1091,14 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0.8453941345214844</v>
+        <v>0.9176483154296875</v>
       </c>
       <c r="K13" t="n">
         <v>500</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0002105236053466797</v>
+        <v>0.000179290771484375</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -1140,14 +1140,14 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0.9025168418884277</v>
+        <v>0.9341843128204346</v>
       </c>
       <c r="K14" t="n">
         <v>500</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1177,7 +1177,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0002820491790771484</v>
+        <v>0.0001761913299560547</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -1189,14 +1189,14 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0.9568495750427246</v>
+        <v>1.047168493270874</v>
       </c>
       <c r="K15" t="n">
         <v>500</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1226,7 +1226,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0005891323089599609</v>
+        <v>0.0001776218414306641</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -1238,14 +1238,14 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0.8104634284973145</v>
+        <v>0.9952075481414795</v>
       </c>
       <c r="K16" t="n">
         <v>500</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1275,7 +1275,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0001809597015380859</v>
+        <v>0.0001752376556396484</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -1287,14 +1287,14 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.8621304035186768</v>
+        <v>0.911548376083374</v>
       </c>
       <c r="K17" t="n">
         <v>500</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0002102851867675781</v>
+        <v>0.0001728534698486328</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1336,14 +1336,14 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0.7817544937133789</v>
+        <v>0.8624086380004883</v>
       </c>
       <c r="K18" t="n">
         <v>500</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1373,7 +1373,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0002012252807617188</v>
+        <v>0.0002133846282958984</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1385,14 +1385,14 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0.9296061992645264</v>
+        <v>0.9367291927337646</v>
       </c>
       <c r="K19" t="n">
         <v>500</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1422,7 +1422,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0001881122589111328</v>
+        <v>0.0001816749572753906</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1434,14 +1434,14 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.829566478729248</v>
+        <v>0.8919174671173096</v>
       </c>
       <c r="K20" t="n">
         <v>500</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1471,7 +1471,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0001916885375976562</v>
+        <v>0.0001780986785888672</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1483,14 +1483,14 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.9262909889221191</v>
+        <v>0.9060139656066895</v>
       </c>
       <c r="K21" t="n">
         <v>500</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -1520,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0002286434173583984</v>
+        <v>0.0002355575561523438</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1532,14 +1532,14 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>1.320345878601074</v>
+        <v>1.371628046035767</v>
       </c>
       <c r="K22" t="n">
         <v>500</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -1569,7 +1569,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0002043247222900391</v>
+        <v>0.0002896785736083984</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1581,14 +1581,14 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>1.23200798034668</v>
+        <v>1.283051490783691</v>
       </c>
       <c r="K23" t="n">
         <v>500</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -1618,7 +1618,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0002138614654541016</v>
+        <v>0.0002853870391845703</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1630,14 +1630,14 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>1.439387559890747</v>
+        <v>1.191197395324707</v>
       </c>
       <c r="K24" t="n">
         <v>500</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -1667,7 +1667,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0002157688140869141</v>
+        <v>0.0003046989440917969</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1679,14 +1679,14 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>1.121364593505859</v>
+        <v>1.105425596237183</v>
       </c>
       <c r="K25" t="n">
         <v>500</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0002183914184570312</v>
+        <v>0.0002310276031494141</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -1728,14 +1728,14 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>1.297212362289429</v>
+        <v>1.279598712921143</v>
       </c>
       <c r="K26" t="n">
         <v>500</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0002319812774658203</v>
+        <v>0.0002095699310302734</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1777,14 +1777,14 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1.225870132446289</v>
+        <v>1.328072786331177</v>
       </c>
       <c r="K27" t="n">
         <v>500</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -1814,7 +1814,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0003139972686767578</v>
+        <v>0.0002284049987792969</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1826,14 +1826,14 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1.214123725891113</v>
+        <v>1.698895215988159</v>
       </c>
       <c r="K28" t="n">
         <v>500</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -1863,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0002787113189697266</v>
+        <v>0.0002236366271972656</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1875,14 +1875,14 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>1.220446348190308</v>
+        <v>1.471688747406006</v>
       </c>
       <c r="K29" t="n">
         <v>500</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -1912,7 +1912,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0002422332763671875</v>
+        <v>0.0002384185791015625</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1924,14 +1924,14 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>1.196954250335693</v>
+        <v>1.159034729003906</v>
       </c>
       <c r="K30" t="n">
         <v>500</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -1961,7 +1961,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0002491474151611328</v>
+        <v>0.0002129077911376953</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -1973,14 +1973,14 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>1.084012985229492</v>
+        <v>1.095954179763794</v>
       </c>
       <c r="K31" t="n">
         <v>500</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2010,7 +2010,7 @@
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0004701614379882812</v>
+        <v>0.0004694461822509766</v>
       </c>
       <c r="G32" t="n">
         <v>9</v>
@@ -2022,14 +2022,14 @@
         <v>9</v>
       </c>
       <c r="J32" t="n">
-        <v>14.41273069381714</v>
+        <v>14.71124267578125</v>
       </c>
       <c r="K32" t="n">
         <v>791</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2059,7 +2059,7 @@
         <v>16</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0004472732543945312</v>
+        <v>0.0004351139068603516</v>
       </c>
       <c r="G33" t="n">
         <v>10</v>
@@ -2071,14 +2071,14 @@
         <v>10</v>
       </c>
       <c r="J33" t="n">
-        <v>12.82056999206543</v>
+        <v>11.44601488113403</v>
       </c>
       <c r="K33" t="n">
         <v>577</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2108,7 +2108,7 @@
         <v>16</v>
       </c>
       <c r="F34" t="n">
-        <v>0.0004253387451171875</v>
+        <v>0.000431060791015625</v>
       </c>
       <c r="G34" t="n">
         <v>11</v>
@@ -2120,14 +2120,14 @@
         <v>11</v>
       </c>
       <c r="J34" t="n">
-        <v>10.85699009895325</v>
+        <v>11.08603596687317</v>
       </c>
       <c r="K34" t="n">
         <v>596</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2157,7 +2157,7 @@
         <v>14</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0004503726959228516</v>
+        <v>0.0004327297210693359</v>
       </c>
       <c r="G35" t="n">
         <v>10</v>
@@ -2169,14 +2169,14 @@
         <v>10</v>
       </c>
       <c r="J35" t="n">
-        <v>14.3402693271637</v>
+        <v>14.2828676700592</v>
       </c>
       <c r="K35" t="n">
         <v>740</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2206,7 +2206,7 @@
         <v>16</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0004658699035644531</v>
+        <v>0.0004262924194335938</v>
       </c>
       <c r="G36" t="n">
         <v>10</v>
@@ -2218,14 +2218,14 @@
         <v>10</v>
       </c>
       <c r="J36" t="n">
-        <v>13.64732885360718</v>
+        <v>14.45707964897156</v>
       </c>
       <c r="K36" t="n">
         <v>693</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -2255,7 +2255,7 @@
         <v>14</v>
       </c>
       <c r="F37" t="n">
-        <v>0.0005023479461669922</v>
+        <v>0.0004372596740722656</v>
       </c>
       <c r="G37" t="n">
         <v>9</v>
@@ -2267,14 +2267,14 @@
         <v>9</v>
       </c>
       <c r="J37" t="n">
-        <v>18.62365484237671</v>
+        <v>18.26830053329468</v>
       </c>
       <c r="K37" t="n">
         <v>1044</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -2304,7 +2304,7 @@
         <v>14</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0004506111145019531</v>
+        <v>0.0004308223724365234</v>
       </c>
       <c r="G38" t="n">
         <v>10</v>
@@ -2316,14 +2316,14 @@
         <v>10</v>
       </c>
       <c r="J38" t="n">
-        <v>10.53196287155151</v>
+        <v>11.06036329269409</v>
       </c>
       <c r="K38" t="n">
         <v>533</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -2353,7 +2353,7 @@
         <v>16</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0004589557647705078</v>
+        <v>0.0005018711090087891</v>
       </c>
       <c r="G39" t="n">
         <v>10</v>
@@ -2365,14 +2365,14 @@
         <v>10</v>
       </c>
       <c r="J39" t="n">
-        <v>11.27620911598206</v>
+        <v>11.51526045799255</v>
       </c>
       <c r="K39" t="n">
         <v>573</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -2402,7 +2402,7 @@
         <v>15</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0004260540008544922</v>
+        <v>0.0004415512084960938</v>
       </c>
       <c r="G40" t="n">
         <v>10</v>
@@ -2414,14 +2414,14 @@
         <v>10</v>
       </c>
       <c r="J40" t="n">
-        <v>11.93673515319824</v>
+        <v>11.60809350013733</v>
       </c>
       <c r="K40" t="n">
         <v>608</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -2451,7 +2451,7 @@
         <v>16</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0004470348358154297</v>
+        <v>0.0007634162902832031</v>
       </c>
       <c r="G41" t="n">
         <v>9</v>
@@ -2463,14 +2463,14 @@
         <v>9</v>
       </c>
       <c r="J41" t="n">
-        <v>14.22837615013123</v>
+        <v>14.06311774253845</v>
       </c>
       <c r="K41" t="n">
         <v>700</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -2500,7 +2500,7 @@
         <v>29</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0006692409515380859</v>
+        <v>0.0006697177886962891</v>
       </c>
       <c r="G42" t="n">
         <v>21</v>
@@ -2512,14 +2512,14 @@
         <v>21</v>
       </c>
       <c r="J42" t="n">
-        <v>43.50261116027832</v>
+        <v>42.26665210723877</v>
       </c>
       <c r="K42" t="n">
         <v>747</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -2549,7 +2549,7 @@
         <v>35</v>
       </c>
       <c r="F43" t="n">
-        <v>0.0006241798400878906</v>
+        <v>0.0007543563842773438</v>
       </c>
       <c r="G43" t="n">
         <v>20</v>
@@ -2561,14 +2561,14 @@
         <v>20</v>
       </c>
       <c r="J43" t="n">
-        <v>61.45580530166626</v>
+        <v>62.27810668945312</v>
       </c>
       <c r="K43" t="n">
         <v>1116</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -2598,7 +2598,7 @@
         <v>29</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0006153583526611328</v>
+        <v>0.0006077289581298828</v>
       </c>
       <c r="G44" t="n">
         <v>19</v>
@@ -2610,14 +2610,14 @@
         <v>19</v>
       </c>
       <c r="J44" t="n">
-        <v>70.93242430686951</v>
+        <v>69.95350241661072</v>
       </c>
       <c r="K44" t="n">
         <v>1340</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -2647,7 +2647,7 @@
         <v>30</v>
       </c>
       <c r="F45" t="n">
-        <v>0.0007596015930175781</v>
+        <v>0.0006875991821289062</v>
       </c>
       <c r="G45" t="n">
         <v>21</v>
@@ -2659,14 +2659,14 @@
         <v>21</v>
       </c>
       <c r="J45" t="n">
-        <v>40.37636923789978</v>
+        <v>39.7953794002533</v>
       </c>
       <c r="K45" t="n">
         <v>703</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -2696,7 +2696,7 @@
         <v>34</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0006029605865478516</v>
+        <v>0.0006520748138427734</v>
       </c>
       <c r="G46" t="n">
         <v>21</v>
@@ -2708,14 +2708,14 @@
         <v>21</v>
       </c>
       <c r="J46" t="n">
-        <v>46.64588117599487</v>
+        <v>45.94612050056458</v>
       </c>
       <c r="K46" t="n">
         <v>930</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -2745,7 +2745,7 @@
         <v>30</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0006453990936279297</v>
+        <v>0.0007145404815673828</v>
       </c>
       <c r="G47" t="n">
         <v>20</v>
@@ -2757,14 +2757,14 @@
         <v>20</v>
       </c>
       <c r="J47" t="n">
-        <v>83.86033368110657</v>
+        <v>81.08644723892212</v>
       </c>
       <c r="K47" t="n">
         <v>1304</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -2794,7 +2794,7 @@
         <v>32</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0006301403045654297</v>
+        <v>0.0006103515625</v>
       </c>
       <c r="G48" t="n">
         <v>20</v>
@@ -2806,14 +2806,14 @@
         <v>20</v>
       </c>
       <c r="J48" t="n">
-        <v>75.06829524040222</v>
+        <v>74.66631174087524</v>
       </c>
       <c r="K48" t="n">
         <v>1202</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -2843,7 +2843,7 @@
         <v>33</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0006315708160400391</v>
+        <v>0.002091646194458008</v>
       </c>
       <c r="G49" t="n">
         <v>20</v>
@@ -2855,14 +2855,14 @@
         <v>20</v>
       </c>
       <c r="J49" t="n">
-        <v>53.43622255325317</v>
+        <v>53.50800895690918</v>
       </c>
       <c r="K49" t="n">
         <v>809</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M49" t="n">
@@ -2892,7 +2892,7 @@
         <v>28</v>
       </c>
       <c r="F50" t="n">
-        <v>0.0006034374237060547</v>
+        <v>0.0006411075592041016</v>
       </c>
       <c r="G50" t="n">
         <v>20</v>
@@ -2904,14 +2904,14 @@
         <v>20</v>
       </c>
       <c r="J50" t="n">
-        <v>50.50098752975464</v>
+        <v>50.38291645050049</v>
       </c>
       <c r="K50" t="n">
         <v>809</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M50" t="n">
@@ -2941,7 +2941,7 @@
         <v>35</v>
       </c>
       <c r="F51" t="n">
-        <v>0.00063323974609375</v>
+        <v>0.0007753372192382812</v>
       </c>
       <c r="G51" t="n">
         <v>20</v>
@@ -2953,14 +2953,14 @@
         <v>20</v>
       </c>
       <c r="J51" t="n">
-        <v>50.09514379501343</v>
+        <v>49.42272329330444</v>
       </c>
       <c r="K51" t="n">
         <v>851</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M51" t="n">
@@ -2990,7 +2990,7 @@
         <v>54</v>
       </c>
       <c r="F52" t="n">
-        <v>0.0008711814880371094</v>
+        <v>0.0008676052093505859</v>
       </c>
       <c r="G52" t="n">
         <v>34</v>
@@ -3002,14 +3002,14 @@
         <v>34</v>
       </c>
       <c r="J52" t="n">
-        <v>188.9952800273895</v>
+        <v>179.1821780204773</v>
       </c>
       <c r="K52" t="n">
         <v>1480</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M52" t="n">
@@ -3039,7 +3039,7 @@
         <v>59</v>
       </c>
       <c r="F53" t="n">
-        <v>0.0009224414825439453</v>
+        <v>0.0008320808410644531</v>
       </c>
       <c r="G53" t="n">
         <v>34</v>
@@ -3051,14 +3051,14 @@
         <v>34</v>
       </c>
       <c r="J53" t="n">
-        <v>245.5376000404358</v>
+        <v>236.1913599967957</v>
       </c>
       <c r="K53" t="n">
         <v>1809</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M53" t="n">
@@ -3088,7 +3088,7 @@
         <v>54</v>
       </c>
       <c r="F54" t="n">
-        <v>0.0008656978607177734</v>
+        <v>0.0009226799011230469</v>
       </c>
       <c r="G54" t="n">
         <v>32</v>
@@ -3100,14 +3100,14 @@
         <v>32</v>
       </c>
       <c r="J54" t="n">
-        <v>205.4348886013031</v>
+        <v>207.8382818698883</v>
       </c>
       <c r="K54" t="n">
         <v>1544</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M54" t="n">
@@ -3137,7 +3137,7 @@
         <v>53</v>
       </c>
       <c r="F55" t="n">
-        <v>0.0008401870727539062</v>
+        <v>0.0008869171142578125</v>
       </c>
       <c r="G55" t="n">
         <v>33</v>
@@ -3149,14 +3149,14 @@
         <v>33</v>
       </c>
       <c r="J55" t="n">
-        <v>244.4579713344574</v>
+        <v>239.0668163299561</v>
       </c>
       <c r="K55" t="n">
         <v>1726</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M55" t="n">
@@ -3186,7 +3186,7 @@
         <v>56</v>
       </c>
       <c r="F56" t="n">
-        <v>0.0008304119110107422</v>
+        <v>0.0009202957153320312</v>
       </c>
       <c r="G56" t="n">
         <v>33</v>
@@ -3198,14 +3198,14 @@
         <v>33</v>
       </c>
       <c r="J56" t="n">
-        <v>237.232170343399</v>
+        <v>228.8066704273224</v>
       </c>
       <c r="K56" t="n">
         <v>1839</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M56" t="n">
@@ -3235,7 +3235,7 @@
         <v>51</v>
       </c>
       <c r="F57" t="n">
-        <v>0.0008215904235839844</v>
+        <v>0.0009779930114746094</v>
       </c>
       <c r="G57" t="n">
         <v>37</v>
@@ -3247,14 +3247,14 @@
         <v>37</v>
       </c>
       <c r="J57" t="n">
-        <v>94.84594464302063</v>
+        <v>92.53922843933105</v>
       </c>
       <c r="K57" t="n">
         <v>693</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M57" t="n">
@@ -3284,7 +3284,7 @@
         <v>56</v>
       </c>
       <c r="F58" t="n">
-        <v>0.00092315673828125</v>
+        <v>0.0008664131164550781</v>
       </c>
       <c r="G58" t="n">
         <v>33</v>
@@ -3296,14 +3296,14 @@
         <v>33</v>
       </c>
       <c r="J58" t="n">
-        <v>273.2515223026276</v>
+        <v>214.8710596561432</v>
       </c>
       <c r="K58" t="n">
         <v>1727</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M58" t="n">
@@ -3333,7 +3333,7 @@
         <v>54</v>
       </c>
       <c r="F59" t="n">
-        <v>0.001594066619873047</v>
+        <v>0.0009298324584960938</v>
       </c>
       <c r="G59" t="n">
         <v>33</v>
@@ -3345,21 +3345,21 @@
         <v>33</v>
       </c>
       <c r="J59" t="n">
-        <v>325.9298918247223</v>
+        <v>1913.283223628998</v>
       </c>
       <c r="K59" t="n">
-        <v>1694</v>
+        <v>1293</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="M59" t="n">
-        <v>4691</v>
+        <v>3588</v>
       </c>
       <c r="N59" t="n">
-        <v>957555</v>
+        <v>710836</v>
       </c>
       <c r="O59" t="n">
         <v>-38.88888888888889</v>
@@ -3382,7 +3382,7 @@
         <v>49</v>
       </c>
       <c r="F60" t="n">
-        <v>0.001333713531494141</v>
+        <v>0.001736640930175781</v>
       </c>
       <c r="G60" t="n">
         <v>33</v>
@@ -3394,14 +3394,14 @@
         <v>33</v>
       </c>
       <c r="J60" t="n">
-        <v>225.7591922283173</v>
+        <v>163.1052947044373</v>
       </c>
       <c r="K60" t="n">
         <v>1030</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -3431,7 +3431,7 @@
         <v>55</v>
       </c>
       <c r="F61" t="n">
-        <v>0.001450538635253906</v>
+        <v>0.00086212158203125</v>
       </c>
       <c r="G61" t="n">
         <v>33</v>
@@ -3443,14 +3443,14 @@
         <v>33</v>
       </c>
       <c r="J61" t="n">
-        <v>220.2865962982178</v>
+        <v>151.0003099441528</v>
       </c>
       <c r="K61" t="n">
         <v>1189</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M61" t="n">
@@ -3480,36 +3480,36 @@
         <v>59</v>
       </c>
       <c r="F62" t="n">
-        <v>0.001456737518310547</v>
+        <v>0.001312255859375</v>
       </c>
       <c r="G62" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="J62" t="n">
-        <v>672.926008939743</v>
+        <v>363.4724988937378</v>
       </c>
       <c r="K62" t="n">
-        <v>39</v>
+        <v>2000</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>time_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M62" t="n">
-        <v>63</v>
+        <v>8810</v>
       </c>
       <c r="N62" t="n">
-        <v>18102</v>
+        <v>1160085</v>
       </c>
       <c r="O62" t="n">
-        <v>-5.084745762711865</v>
+        <v>-37.28813559322034</v>
       </c>
     </row>
     <row r="63">
@@ -3529,7 +3529,7 @@
         <v>65</v>
       </c>
       <c r="F63" t="n">
-        <v>0.001516819000244141</v>
+        <v>0.001702547073364258</v>
       </c>
       <c r="G63" t="n">
         <v>42</v>
@@ -3541,14 +3541,14 @@
         <v>42</v>
       </c>
       <c r="J63" t="n">
-        <v>258.5089955329895</v>
+        <v>225.4998164176941</v>
       </c>
       <c r="K63" t="n">
         <v>1190</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M63" t="n">
@@ -3578,7 +3578,7 @@
         <v>65</v>
       </c>
       <c r="F64" t="n">
-        <v>0.001379728317260742</v>
+        <v>0.0009648799896240234</v>
       </c>
       <c r="G64" t="n">
         <v>39</v>
@@ -3590,14 +3590,14 @@
         <v>39</v>
       </c>
       <c r="J64" t="n">
-        <v>458.6520426273346</v>
+        <v>401.0946478843689</v>
       </c>
       <c r="K64" t="n">
         <v>2000</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>iteration_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M64" t="n">
@@ -3627,7 +3627,7 @@
         <v>62</v>
       </c>
       <c r="F65" t="n">
-        <v>0.002218008041381836</v>
+        <v>0.001374244689941406</v>
       </c>
       <c r="G65" t="n">
         <v>39</v>
@@ -3639,14 +3639,14 @@
         <v>39</v>
       </c>
       <c r="J65" t="n">
-        <v>445.1842617988586</v>
+        <v>379.9831991195679</v>
       </c>
       <c r="K65" t="n">
         <v>1869</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M65" t="n">
@@ -3676,7 +3676,7 @@
         <v>62</v>
       </c>
       <c r="F66" t="n">
-        <v>0.001027822494506836</v>
+        <v>0.0009961128234863281</v>
       </c>
       <c r="G66" t="n">
         <v>42</v>
@@ -3688,14 +3688,14 @@
         <v>42</v>
       </c>
       <c r="J66" t="n">
-        <v>275.5020015239716</v>
+        <v>227.5224435329437</v>
       </c>
       <c r="K66" t="n">
         <v>1371</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M66" t="n">
@@ -3725,7 +3725,7 @@
         <v>58</v>
       </c>
       <c r="F67" t="n">
-        <v>0.0016632080078125</v>
+        <v>0.001064777374267578</v>
       </c>
       <c r="G67" t="n">
         <v>36</v>
@@ -3737,14 +3737,14 @@
         <v>36</v>
       </c>
       <c r="J67" t="n">
-        <v>487.7747313976288</v>
+        <v>366.2641031742096</v>
       </c>
       <c r="K67" t="n">
         <v>1974</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M67" t="n">
@@ -3774,7 +3774,7 @@
         <v>61</v>
       </c>
       <c r="F68" t="n">
-        <v>0.002142667770385742</v>
+        <v>0.001018285751342773</v>
       </c>
       <c r="G68" t="n">
         <v>38</v>
@@ -3786,14 +3786,14 @@
         <v>38</v>
       </c>
       <c r="J68" t="n">
-        <v>501.3931684494019</v>
+        <v>390.7152700424194</v>
       </c>
       <c r="K68" t="n">
         <v>2000</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>iteration_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M68" t="n">
@@ -3823,36 +3823,36 @@
         <v>60</v>
       </c>
       <c r="F69" t="n">
-        <v>0.002043485641479492</v>
+        <v>0.005270481109619141</v>
       </c>
       <c r="G69" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J69" t="n">
-        <v>600.3502252101898</v>
+        <v>433.4855642318726</v>
       </c>
       <c r="K69" t="n">
-        <v>1316</v>
+        <v>1976</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>time_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M69" t="n">
-        <v>3746</v>
+        <v>7271</v>
       </c>
       <c r="N69" t="n">
-        <v>789026</v>
+        <v>1126151</v>
       </c>
       <c r="O69" t="n">
-        <v>-33.33333333333333</v>
+        <v>-38.33333333333334</v>
       </c>
     </row>
     <row r="70">
@@ -3872,7 +3872,7 @@
         <v>66</v>
       </c>
       <c r="F70" t="n">
-        <v>0.004863500595092773</v>
+        <v>0.001591682434082031</v>
       </c>
       <c r="G70" t="n">
         <v>38</v>
@@ -3884,21 +3884,21 @@
         <v>38</v>
       </c>
       <c r="J70" t="n">
-        <v>600.1720998287201</v>
+        <v>510.2898092269897</v>
       </c>
       <c r="K70" t="n">
-        <v>1956</v>
+        <v>2000</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>time_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M70" t="n">
-        <v>4672</v>
+        <v>4942</v>
       </c>
       <c r="N70" t="n">
-        <v>1207170</v>
+        <v>1226138</v>
       </c>
       <c r="O70" t="n">
         <v>-42.42424242424242</v>
@@ -3921,7 +3921,7 @@
         <v>66</v>
       </c>
       <c r="F71" t="n">
-        <v>0.002317190170288086</v>
+        <v>0.002067327499389648</v>
       </c>
       <c r="G71" t="n">
         <v>41</v>
@@ -3933,14 +3933,14 @@
         <v>41</v>
       </c>
       <c r="J71" t="n">
-        <v>580.1826455593109</v>
+        <v>403.1454524993896</v>
       </c>
       <c r="K71" t="n">
         <v>1369</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M71" t="n">
@@ -3978,7 +3978,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
@@ -4086,7 +4086,7 @@
         <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0002939701080322266</v>
+        <v>0.0004546642303466797</v>
       </c>
       <c r="G2" t="n">
         <v>10</v>
@@ -4098,14 +4098,14 @@
         <v>10</v>
       </c>
       <c r="J2" t="n">
-        <v>3.121384382247925</v>
+        <v>4.258242845535278</v>
       </c>
       <c r="K2" t="n">
         <v>621</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4142,7 +4142,7 @@
         <v>13</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0001797676086425781</v>
+        <v>0.0002226829528808594</v>
       </c>
       <c r="G3" t="n">
         <v>9</v>
@@ -4154,14 +4154,14 @@
         <v>9</v>
       </c>
       <c r="J3" t="n">
-        <v>5.132656097412109</v>
+        <v>6.767327070236206</v>
       </c>
       <c r="K3" t="n">
         <v>1057</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4198,7 +4198,7 @@
         <v>13</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0001692771911621094</v>
+        <v>0.0002655982971191406</v>
       </c>
       <c r="G4" t="n">
         <v>10</v>
@@ -4210,14 +4210,14 @@
         <v>10</v>
       </c>
       <c r="J4" t="n">
-        <v>2.873636245727539</v>
+        <v>3.186977386474609</v>
       </c>
       <c r="K4" t="n">
         <v>581</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4254,7 +4254,7 @@
         <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0001795291900634766</v>
+        <v>0.0007295608520507812</v>
       </c>
       <c r="G5" t="n">
         <v>10</v>
@@ -4266,14 +4266,14 @@
         <v>10</v>
       </c>
       <c r="J5" t="n">
-        <v>3.999540328979492</v>
+        <v>5.360579490661621</v>
       </c>
       <c r="K5" t="n">
         <v>771</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -4310,7 +4310,7 @@
         <v>13</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0001714229583740234</v>
+        <v>0.000270843505859375</v>
       </c>
       <c r="G6" t="n">
         <v>10</v>
@@ -4322,14 +4322,14 @@
         <v>10</v>
       </c>
       <c r="J6" t="n">
-        <v>7.847492456436157</v>
+        <v>3.776985645294189</v>
       </c>
       <c r="K6" t="n">
         <v>711</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -4366,7 +4366,7 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0002188682556152344</v>
+        <v>0.0005857944488525391</v>
       </c>
       <c r="G7" t="n">
         <v>11</v>
@@ -4378,14 +4378,14 @@
         <v>11</v>
       </c>
       <c r="J7" t="n">
-        <v>2.306689977645874</v>
+        <v>2.980002641677856</v>
       </c>
       <c r="K7" t="n">
         <v>533</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -4422,7 +4422,7 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0002839565277099609</v>
+        <v>0.0004811286926269531</v>
       </c>
       <c r="G8" t="n">
         <v>11</v>
@@ -4434,14 +4434,14 @@
         <v>11</v>
       </c>
       <c r="J8" t="n">
-        <v>2.653379678726196</v>
+        <v>11.80047678947449</v>
       </c>
       <c r="K8" t="n">
         <v>587</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -4478,7 +4478,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0001652240753173828</v>
+        <v>0.0006129741668701172</v>
       </c>
       <c r="G9" t="n">
         <v>11</v>
@@ -4490,14 +4490,14 @@
         <v>11</v>
       </c>
       <c r="J9" t="n">
-        <v>2.591329097747803</v>
+        <v>2.994483470916748</v>
       </c>
       <c r="K9" t="n">
         <v>503</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -4534,7 +4534,7 @@
         <v>13</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0001680850982666016</v>
+        <v>0.0001845359802246094</v>
       </c>
       <c r="G10" t="n">
         <v>10</v>
@@ -4546,14 +4546,14 @@
         <v>10</v>
       </c>
       <c r="J10" t="n">
-        <v>3.680405855178833</v>
+        <v>3.959414482116699</v>
       </c>
       <c r="K10" t="n">
         <v>558</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -4590,7 +4590,7 @@
         <v>13</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0001678466796875</v>
+        <v>0.0004184246063232422</v>
       </c>
       <c r="G11" t="n">
         <v>10</v>
@@ -4602,14 +4602,14 @@
         <v>10</v>
       </c>
       <c r="J11" t="n">
-        <v>3.513470649719238</v>
+        <v>4.496594190597534</v>
       </c>
       <c r="K11" t="n">
         <v>757</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -4646,7 +4646,7 @@
         <v>23</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0003120899200439453</v>
+        <v>0.0002965927124023438</v>
       </c>
       <c r="G12" t="n">
         <v>18</v>
@@ -4658,14 +4658,14 @@
         <v>18</v>
       </c>
       <c r="J12" t="n">
-        <v>8.711171388626099</v>
+        <v>10.7136697769165</v>
       </c>
       <c r="K12" t="n">
         <v>715</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -4702,7 +4702,7 @@
         <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0002231597900390625</v>
+        <v>0.0004634857177734375</v>
       </c>
       <c r="G13" t="n">
         <v>19</v>
@@ -4714,14 +4714,14 @@
         <v>19</v>
       </c>
       <c r="J13" t="n">
-        <v>11.22806763648987</v>
+        <v>13.91252970695496</v>
       </c>
       <c r="K13" t="n">
         <v>1093</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -4758,7 +4758,7 @@
         <v>26</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0002179145812988281</v>
+        <v>0.0005500316619873047</v>
       </c>
       <c r="G14" t="n">
         <v>17</v>
@@ -4770,14 +4770,14 @@
         <v>17</v>
       </c>
       <c r="J14" t="n">
-        <v>5.541896343231201</v>
+        <v>7.505527496337891</v>
       </c>
       <c r="K14" t="n">
         <v>643</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -4814,7 +4814,7 @@
         <v>26</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0002279281616210938</v>
+        <v>0.0003905296325683594</v>
       </c>
       <c r="G15" t="n">
         <v>18</v>
@@ -4826,14 +4826,14 @@
         <v>18</v>
       </c>
       <c r="J15" t="n">
-        <v>8.037664651870728</v>
+        <v>10.29904842376709</v>
       </c>
       <c r="K15" t="n">
         <v>716</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -4870,7 +4870,7 @@
         <v>25</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0002272129058837891</v>
+        <v>0.0003018379211425781</v>
       </c>
       <c r="G16" t="n">
         <v>19</v>
@@ -4882,14 +4882,14 @@
         <v>19</v>
       </c>
       <c r="J16" t="n">
-        <v>6.237082481384277</v>
+        <v>8.820015668869019</v>
       </c>
       <c r="K16" t="n">
         <v>557</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -4926,7 +4926,7 @@
         <v>25</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0002677440643310547</v>
+        <v>0.0006895065307617188</v>
       </c>
       <c r="G17" t="n">
         <v>18</v>
@@ -4938,14 +4938,14 @@
         <v>18</v>
       </c>
       <c r="J17" t="n">
-        <v>8.159197807312012</v>
+        <v>10.17579555511475</v>
       </c>
       <c r="K17" t="n">
         <v>718</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -4982,7 +4982,7 @@
         <v>27</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0002274513244628906</v>
+        <v>0.0006136894226074219</v>
       </c>
       <c r="G18" t="n">
         <v>16</v>
@@ -4994,14 +4994,14 @@
         <v>16</v>
       </c>
       <c r="J18" t="n">
-        <v>8.067476272583008</v>
+        <v>10.45434665679932</v>
       </c>
       <c r="K18" t="n">
         <v>941</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -5038,7 +5038,7 @@
         <v>25</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0002279281616210938</v>
+        <v>0.0003392696380615234</v>
       </c>
       <c r="G19" t="n">
         <v>19</v>
@@ -5050,14 +5050,14 @@
         <v>19</v>
       </c>
       <c r="J19" t="n">
-        <v>5.989822864532471</v>
+        <v>7.862460851669312</v>
       </c>
       <c r="K19" t="n">
         <v>577</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -5094,7 +5094,7 @@
         <v>25</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0002186298370361328</v>
+        <v>0.0004987716674804688</v>
       </c>
       <c r="G20" t="n">
         <v>18</v>
@@ -5106,14 +5106,14 @@
         <v>18</v>
       </c>
       <c r="J20" t="n">
-        <v>6.231969833374023</v>
+        <v>8.525230407714844</v>
       </c>
       <c r="K20" t="n">
         <v>584</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -5150,7 +5150,7 @@
         <v>24</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0002253055572509766</v>
+        <v>0.0003387928009033203</v>
       </c>
       <c r="G21" t="n">
         <v>17</v>
@@ -5162,14 +5162,14 @@
         <v>17</v>
       </c>
       <c r="J21" t="n">
-        <v>5.434717416763306</v>
+        <v>7.243110418319702</v>
       </c>
       <c r="K21" t="n">
         <v>592</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -5206,7 +5206,7 @@
         <v>59</v>
       </c>
       <c r="F22" t="n">
-        <v>0.001678466796875</v>
+        <v>0.002276420593261719</v>
       </c>
       <c r="G22" t="n">
         <v>48</v>
@@ -5218,14 +5218,14 @@
         <v>48</v>
       </c>
       <c r="J22" t="n">
-        <v>141.1046724319458</v>
+        <v>168.2846426963806</v>
       </c>
       <c r="K22" t="n">
         <v>673</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -5262,36 +5262,36 @@
         <v>65</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0009593963623046875</v>
+        <v>0.001277923583984375</v>
       </c>
       <c r="G23" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>334.5407745838165</v>
+        <v>600.0040786266327</v>
       </c>
       <c r="K23" t="n">
-        <v>1811</v>
+        <v>674</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="M23" t="n">
-        <v>5857</v>
+        <v>1562</v>
       </c>
       <c r="N23" t="n">
-        <v>1035668</v>
+        <v>392162</v>
       </c>
       <c r="O23" t="n">
-        <v>-40</v>
+        <v>-30.76923076923077</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -5318,7 +5318,7 @@
         <v>65</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0009922981262207031</v>
+        <v>0.00103449821472168</v>
       </c>
       <c r="G24" t="n">
         <v>40</v>
@@ -5330,14 +5330,14 @@
         <v>40</v>
       </c>
       <c r="J24" t="n">
-        <v>403.3696093559265</v>
+        <v>377.0377097129822</v>
       </c>
       <c r="K24" t="n">
         <v>2000</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>iteration_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -5374,7 +5374,7 @@
         <v>62</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0009846687316894531</v>
+        <v>0.00146794319152832</v>
       </c>
       <c r="G25" t="n">
         <v>39</v>
@@ -5386,14 +5386,14 @@
         <v>39</v>
       </c>
       <c r="J25" t="n">
-        <v>372.8304760456085</v>
+        <v>352.7665441036224</v>
       </c>
       <c r="K25" t="n">
         <v>1934</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -5430,7 +5430,7 @@
         <v>64</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0009992122650146484</v>
+        <v>0.001752138137817383</v>
       </c>
       <c r="G26" t="n">
         <v>45</v>
@@ -5442,14 +5442,14 @@
         <v>45</v>
       </c>
       <c r="J26" t="n">
-        <v>132.8972930908203</v>
+        <v>130.66969871521</v>
       </c>
       <c r="K26" t="n">
         <v>568</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -5486,7 +5486,7 @@
         <v>58</v>
       </c>
       <c r="F27" t="n">
-        <v>0.001002311706542969</v>
+        <v>0.001019716262817383</v>
       </c>
       <c r="G27" t="n">
         <v>47</v>
@@ -5498,14 +5498,14 @@
         <v>47</v>
       </c>
       <c r="J27" t="n">
-        <v>139.823650598526</v>
+        <v>135.0059757232666</v>
       </c>
       <c r="K27" t="n">
         <v>595</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -5542,7 +5542,7 @@
         <v>60</v>
       </c>
       <c r="F28" t="n">
-        <v>0.001001834869384766</v>
+        <v>0.0009775161743164062</v>
       </c>
       <c r="G28" t="n">
         <v>38</v>
@@ -5554,14 +5554,14 @@
         <v>38</v>
       </c>
       <c r="J28" t="n">
-        <v>349.5190861225128</v>
+        <v>338.3487229347229</v>
       </c>
       <c r="K28" t="n">
         <v>1768</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -5598,7 +5598,7 @@
         <v>61</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0009927749633789062</v>
+        <v>0.0009698867797851562</v>
       </c>
       <c r="G29" t="n">
         <v>42</v>
@@ -5610,21 +5610,21 @@
         <v>42</v>
       </c>
       <c r="J29" t="n">
-        <v>2725.833329916</v>
+        <v>255.3707990646362</v>
       </c>
       <c r="K29" t="n">
-        <v>825</v>
+        <v>1181</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>time_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>3040</v>
+        <v>5277</v>
       </c>
       <c r="N29" t="n">
-        <v>515792</v>
+        <v>721817</v>
       </c>
       <c r="O29" t="n">
         <v>-31.14754098360656</v>
@@ -5654,7 +5654,7 @@
         <v>65</v>
       </c>
       <c r="F30" t="n">
-        <v>0.001394748687744141</v>
+        <v>0.0009624958038330078</v>
       </c>
       <c r="G30" t="n">
         <v>40</v>
@@ -5666,14 +5666,14 @@
         <v>40</v>
       </c>
       <c r="J30" t="n">
-        <v>445.0826172828674</v>
+        <v>374.4325206279755</v>
       </c>
       <c r="K30" t="n">
         <v>2000</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>iteration_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -5710,7 +5710,7 @@
         <v>66</v>
       </c>
       <c r="F31" t="n">
-        <v>0.004366874694824219</v>
+        <v>0.0009930133819580078</v>
       </c>
       <c r="G31" t="n">
         <v>39</v>
@@ -5722,14 +5722,14 @@
         <v>39</v>
       </c>
       <c r="J31" t="n">
-        <v>292.6419599056244</v>
+        <v>238.309992313385</v>
       </c>
       <c r="K31" t="n">
         <v>1371</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -5766,7 +5766,7 @@
         <v>73</v>
       </c>
       <c r="F32" t="n">
-        <v>0.001328945159912109</v>
+        <v>0.001268386840820312</v>
       </c>
       <c r="G32" t="n">
         <v>47</v>
@@ -5778,14 +5778,14 @@
         <v>47</v>
       </c>
       <c r="J32" t="n">
-        <v>532.3455097675323</v>
+        <v>496.6844303607941</v>
       </c>
       <c r="K32" t="n">
         <v>2000</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>iteration_limit</t>
+          <t>it_lim</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -5822,7 +5822,7 @@
         <v>82</v>
       </c>
       <c r="F33" t="n">
-        <v>0.001550197601318359</v>
+        <v>0.001845598220825195</v>
       </c>
       <c r="G33" t="n">
         <v>55</v>
@@ -5834,14 +5834,14 @@
         <v>55</v>
       </c>
       <c r="J33" t="n">
-        <v>287.5273616313934</v>
+        <v>290.1968517303467</v>
       </c>
       <c r="K33" t="n">
         <v>1035</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -5878,7 +5878,7 @@
         <v>80</v>
       </c>
       <c r="F34" t="n">
-        <v>0.001524925231933594</v>
+        <v>0.002858400344848633</v>
       </c>
       <c r="G34" t="n">
         <v>51</v>
@@ -5890,14 +5890,14 @@
         <v>51</v>
       </c>
       <c r="J34" t="n">
-        <v>319.2118294239044</v>
+        <v>329.0786008834839</v>
       </c>
       <c r="K34" t="n">
         <v>1100</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -5934,7 +5934,7 @@
         <v>77</v>
       </c>
       <c r="F35" t="n">
-        <v>0.001221895217895508</v>
+        <v>0.001463890075683594</v>
       </c>
       <c r="G35" t="n">
         <v>49</v>
@@ -5946,14 +5946,14 @@
         <v>49</v>
       </c>
       <c r="J35" t="n">
-        <v>475.3150599002838</v>
+        <v>575.5968372821808</v>
       </c>
       <c r="K35" t="n">
         <v>1850</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -5990,7 +5990,7 @@
         <v>82</v>
       </c>
       <c r="F36" t="n">
-        <v>0.001210927963256836</v>
+        <v>0.001760005950927734</v>
       </c>
       <c r="G36" t="n">
         <v>49</v>
@@ -6002,14 +6002,14 @@
         <v>49</v>
       </c>
       <c r="J36" t="n">
-        <v>452.0888965129852</v>
+        <v>508.7986831665039</v>
       </c>
       <c r="K36" t="n">
         <v>1478</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -6046,36 +6046,36 @@
         <v>79</v>
       </c>
       <c r="F37" t="n">
-        <v>0.001849651336669922</v>
+        <v>0.003864765167236328</v>
       </c>
       <c r="G37" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="J37" t="n">
-        <v>600.1630113124847</v>
+        <v>603.3597164154053</v>
       </c>
       <c r="K37" t="n">
-        <v>1755</v>
+        <v>850</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>time_limit</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="M37" t="n">
-        <v>33888</v>
+        <v>9359</v>
       </c>
       <c r="N37" t="n">
-        <v>1375761</v>
+        <v>698690</v>
       </c>
       <c r="O37" t="n">
-        <v>-39.24050632911392</v>
+        <v>-32.91139240506329</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
@@ -6102,7 +6102,7 @@
         <v>82</v>
       </c>
       <c r="F38" t="n">
-        <v>0.003571033477783203</v>
+        <v>0.003278970718383789</v>
       </c>
       <c r="G38" t="n">
         <v>50</v>
@@ -6114,21 +6114,21 @@
         <v>50</v>
       </c>
       <c r="J38" t="n">
-        <v>430.8802728652954</v>
+        <v>600.5942499637604</v>
       </c>
       <c r="K38" t="n">
-        <v>1150</v>
+        <v>818</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="M38" t="n">
-        <v>9426</v>
+        <v>3836</v>
       </c>
       <c r="N38" t="n">
-        <v>889075</v>
+        <v>634635</v>
       </c>
       <c r="O38" t="n">
         <v>-39.02439024390244</v>
@@ -6158,36 +6158,36 @@
         <v>79</v>
       </c>
       <c r="F39" t="n">
-        <v>0.001255035400390625</v>
+        <v>0.002925634384155273</v>
       </c>
       <c r="G39" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J39" t="n">
-        <v>598.401547908783</v>
+        <v>602.596408367157</v>
       </c>
       <c r="K39" t="n">
-        <v>1850</v>
+        <v>906</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="M39" t="n">
-        <v>23814</v>
+        <v>11017</v>
       </c>
       <c r="N39" t="n">
-        <v>1337429</v>
+        <v>640460</v>
       </c>
       <c r="O39" t="n">
-        <v>-40.50632911392405</v>
+        <v>-37.9746835443038</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
@@ -6214,7 +6214,7 @@
         <v>82</v>
       </c>
       <c r="F40" t="n">
-        <v>0.003673553466796875</v>
+        <v>0.001981258392333984</v>
       </c>
       <c r="G40" t="n">
         <v>51</v>
@@ -6226,21 +6226,21 @@
         <v>51</v>
       </c>
       <c r="J40" t="n">
-        <v>528.3975644111633</v>
+        <v>601.6012725830078</v>
       </c>
       <c r="K40" t="n">
-        <v>1475</v>
+        <v>1000</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>no_improvement_limit</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>10568</v>
+        <v>5070</v>
       </c>
       <c r="N40" t="n">
-        <v>977487</v>
+        <v>627028</v>
       </c>
       <c r="O40" t="n">
         <v>-37.80487804878049</v>
@@ -6270,7 +6270,7 @@
         <v>79</v>
       </c>
       <c r="F41" t="n">
-        <v>0.003118276596069336</v>
+        <v>0.002028703689575195</v>
       </c>
       <c r="G41" t="n">
         <v>52</v>
@@ -6282,21 +6282,21 @@
         <v>52</v>
       </c>
       <c r="J41" t="n">
-        <v>600.0312559604645</v>
+        <v>528.9853572845459</v>
       </c>
       <c r="K41" t="n">
-        <v>1484</v>
+        <v>1508</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>time_limit</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>14222</v>
+        <v>14276</v>
       </c>
       <c r="N41" t="n">
-        <v>1022300</v>
+        <v>1035518</v>
       </c>
       <c r="O41" t="n">
         <v>-34.17721518987342</v>

</xml_diff>